<commit_message>
Implemented safe loading of tiff files
</commit_message>
<xml_diff>
--- a/RGECO.xlsx
+++ b/RGECO.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -22,7 +22,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Author</author>
+    <author>Unknown Author</author>
   </authors>
   <commentList>
     <comment ref="C1" authorId="0">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -142,6 +142,18 @@
   </si>
   <si>
     <t xml:space="preserve">16x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026.02.04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shaker1_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shaker1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z:\Users\Elli\data\in vivo\20260204_shaker1_1-3_AAVGCamp8m_P9\1</t>
   </si>
 </sst>
 </file>
@@ -224,28 +236,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -438,162 +454,259 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AC2"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AC4"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="16.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="14.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="4.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="106.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="27.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="9.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="7.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="7.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="16.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="8.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="9.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="7.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="6.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="9.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="16.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="13.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="16.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="16.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="11.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="13.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="15.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="0" t="n">
+      <c r="H2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="0" t="n">
+      <c r="J2" s="1" t="n">
         <v>416</v>
       </c>
-      <c r="K2" s="0" t="n">
+      <c r="K2" s="1" t="n">
         <v>1024</v>
       </c>
-      <c r="L2" s="0" t="n">
+      <c r="L2" s="1" t="n">
         <v>235.88</v>
       </c>
-      <c r="M2" s="0" t="n">
+      <c r="M2" s="1" t="n">
         <f aca="false">L2/K2</f>
         <v>0.2303515625</v>
       </c>
-      <c r="N2" s="0" t="n">
+      <c r="N2" s="1" t="n">
         <v>18.884</v>
       </c>
-      <c r="O2" s="0" t="n">
+      <c r="O2" s="1" t="n">
         <v>6965</v>
       </c>
-      <c r="P2" s="0" t="n">
+      <c r="P2" s="1" t="n">
         <f aca="false">O2/N2</f>
         <v>368.830756195721</v>
       </c>
-      <c r="U2" s="0" t="n">
+      <c r="U2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="V2" s="0" t="n">
+      <c r="V2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="W2" s="0" t="n">
+      <c r="W2" s="1" t="n">
         <v>2</v>
       </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>320</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>235.88</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <f aca="false">L3/K3</f>
+        <v>0.2303515625</v>
+      </c>
+      <c r="N3" s="1" t="n">
+        <v>24.48</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>8688</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <f aca="false">O3/N3</f>
+        <v>354.901960784314</v>
+      </c>
+      <c r="U3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="W3" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
+      <c r="K4" s="0"/>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0"/>
+      <c r="N4" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>